<commit_message>
Table II and Table III
</commit_message>
<xml_diff>
--- a/output/tables/table_III_return_predictability.xlsx
+++ b/output/tables/table_III_return_predictability.xlsx
@@ -11,8 +11,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R_t1_Q_Comm_Full" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R_t1_Q_NonComm" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R_t1_Q_NonComm_Full" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R_t2_Q_Comm_Full" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R_t2_Q_NonComm_Full" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -494,10 +492,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0003577981894051034</v>
+        <v>0.0003577981894051035</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0001995661937595646</v>
+        <v>0.0001995661937595645</v>
       </c>
       <c r="D3" t="n">
         <v>1.792879759164898</v>
@@ -506,7 +504,7 @@
         <v>153</v>
       </c>
       <c r="F3" t="n">
-        <v>0.07498072240951026</v>
+        <v>0.07498072240951004</v>
       </c>
     </row>
   </sheetData>
@@ -520,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -562,19 +560,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.00136750056190373</v>
+        <v>0.001012442821039563</v>
       </c>
       <c r="C2" t="n">
-        <v>0.001558887990892368</v>
+        <v>0.001309489677889702</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8772282356995514</v>
+        <v>0.773158305967831</v>
       </c>
       <c r="E2" t="n">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3820190932719181</v>
+        <v>0.4406293812109221</v>
       </c>
     </row>
     <row r="3">
@@ -584,85 +582,41 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0004562866158777032</v>
+        <v>0.0004605444588701624</v>
       </c>
       <c r="C3" t="n">
-        <v>0.000278413708253446</v>
+        <v>0.0002233825607407041</v>
       </c>
       <c r="D3" t="n">
-        <v>1.638879848050929</v>
+        <v>2.061684928953558</v>
       </c>
       <c r="E3" t="n">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1037132994876999</v>
+        <v>0.04094081501048508</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Basis</t>
+          <t>Ret</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02515492855879896</v>
+        <v>0.0139640742729678</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0720664177974517</v>
+        <v>0.03110085560621559</v>
       </c>
       <c r="D4" t="n">
-        <v>0.349052017952368</v>
+        <v>0.4489932511752842</v>
       </c>
       <c r="E4" t="n">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7276283069589755</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>S_v</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>-0.004165561954139163</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.003394682794704111</v>
-      </c>
-      <c r="D5" t="n">
-        <v>-1.227084298019734</v>
-      </c>
-      <c r="E5" t="n">
-        <v>128</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.2220607690673455</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ret</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>-0.01854815780365857</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.03643874380802028</v>
-      </c>
-      <c r="D6" t="n">
-        <v>-0.5090229756925941</v>
-      </c>
-      <c r="E6" t="n">
-        <v>128</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.6116193511940335</v>
+        <v>0.654076014081288</v>
       </c>
     </row>
   </sheetData>
@@ -718,19 +672,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.0009857780021970399</v>
+        <v>0.0009857780021970391</v>
       </c>
       <c r="C2" t="n">
         <v>0.001312585960625891</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7510197669088152</v>
+        <v>0.7510197669088146</v>
       </c>
       <c r="E2" t="n">
         <v>153</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4538018923023839</v>
+        <v>0.4538018923023843</v>
       </c>
     </row>
     <row r="3">
@@ -740,7 +694,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.0003392186381108248</v>
+        <v>-0.0003392186381108249</v>
       </c>
       <c r="C3" t="n">
         <v>0.0002030635624938836</v>
@@ -752,7 +706,7 @@
         <v>153</v>
       </c>
       <c r="F3" t="n">
-        <v>0.09687741247667736</v>
+        <v>0.09687741247667714</v>
       </c>
     </row>
   </sheetData>
@@ -766,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,19 +762,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.001278787414207997</v>
+        <v>0.0009577636006659527</v>
       </c>
       <c r="C2" t="n">
-        <v>0.001535620350343818</v>
+        <v>0.001303061314900069</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8327497183282851</v>
+        <v>0.7350103864754847</v>
       </c>
       <c r="E2" t="n">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4065491806427768</v>
+        <v>0.4634656801471708</v>
       </c>
     </row>
     <row r="3">
@@ -830,397 +784,41 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.0003587096667567945</v>
+        <v>-0.0003776220626506965</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0002922994715452766</v>
+        <v>0.000246728518871508</v>
       </c>
       <c r="D3" t="n">
-        <v>-1.227199162764244</v>
+        <v>-1.53051647364428</v>
       </c>
       <c r="E3" t="n">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2220177522040436</v>
+        <v>0.127967473141577</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Basis</t>
+          <t>Ret</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02347315293078273</v>
+        <v>0.00839777130297043</v>
       </c>
       <c r="C4" t="n">
-        <v>0.07245350381077069</v>
+        <v>0.03150739640804179</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3239754007216597</v>
+        <v>0.2665333305936706</v>
       </c>
       <c r="E4" t="n">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="F4" t="n">
-        <v>0.746489594042639</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>S_v</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>-0.00365249216688758</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.003313022824455728</v>
-      </c>
-      <c r="D5" t="n">
-        <v>-1.102465138460862</v>
-      </c>
-      <c r="E5" t="n">
-        <v>128</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.2723443229589753</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ret</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>-0.02065243647787309</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.03628004043369595</v>
-      </c>
-      <c r="D6" t="n">
-        <v>-0.5692506466638788</v>
-      </c>
-      <c r="E6" t="n">
-        <v>128</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.5701914766100749</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Coefficient</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Std_Error</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>t_stat</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>N_months</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>p_value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>const</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.0008745742239192069</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.001564552509791027</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.5589932063296627</v>
-      </c>
-      <c r="E2" t="n">
-        <v>127</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.5771585269375135</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Q_Comm</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.0003814694699642272</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.0003206739323209783</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1.189586778080844</v>
-      </c>
-      <c r="E3" t="n">
-        <v>127</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.2364456402688748</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Basis</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>-0.1348854468659074</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.06874841533060062</v>
-      </c>
-      <c r="D4" t="n">
-        <v>-1.962015360168869</v>
-      </c>
-      <c r="E4" t="n">
-        <v>127</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.05196511587644315</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>S_v</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>-0.001478292107600891</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.003350885524773794</v>
-      </c>
-      <c r="D5" t="n">
-        <v>-0.4411646105698241</v>
-      </c>
-      <c r="E5" t="n">
-        <v>127</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.6598499133555067</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ret</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0.04008231453565547</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.03410292663162661</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1.175333570887246</v>
-      </c>
-      <c r="E6" t="n">
-        <v>127</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.2420774822817708</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Coefficient</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Std_Error</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>t_stat</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>N_months</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>p_value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>const</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.0006044817855793463</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.001552741476365589</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.3892996965561977</v>
-      </c>
-      <c r="E2" t="n">
-        <v>127</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.6977116295825945</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Q_NonComm</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>-0.0004697353334373075</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.0003214227344236432</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-1.461425353995603</v>
-      </c>
-      <c r="E3" t="n">
-        <v>127</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.146388174704247</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Basis</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>-0.1366987884153907</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.06791457455158625</v>
-      </c>
-      <c r="D4" t="n">
-        <v>-2.012804899654605</v>
-      </c>
-      <c r="E4" t="n">
-        <v>127</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.04626656912270244</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>S_v</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>-0.001330545913148971</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.003350131207432538</v>
-      </c>
-      <c r="D5" t="n">
-        <v>-0.397162329104319</v>
-      </c>
-      <c r="E5" t="n">
-        <v>127</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.691919716265107</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ret</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0.04483786802389659</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.03379161481257681</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1.32689332168904</v>
-      </c>
-      <c r="E6" t="n">
-        <v>127</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.1869435988844375</v>
+        <v>0.7901897267441818</v>
       </c>
     </row>
   </sheetData>

</xml_diff>